<commit_message>
Some modify to skills and levels
</commit_message>
<xml_diff>
--- a/Src/Assets/StreamingAssets/Common/Tables/Tables/Skill&Buff.xlsx
+++ b/Src/Assets/StreamingAssets/Common/Tables/Tables/Skill&Buff.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\Common\Tables\Tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CCA\Src\Assets\StreamingAssets\Common\Tables\Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DBB84D-551E-495C-A1B5-59B48C8D82A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8540D561-90AD-49DE-A00B-1D3C15379C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TableExplanation" sheetId="5" r:id="rId1"/>
@@ -1513,30 +1513,9 @@
     <t>丝线编织成茧，我将重新归来</t>
   </si>
   <si>
-    <t>你每受到或进行一次攻击，你获得1点“记忆灵丝”。当你生命值≤0时，若“记忆灵丝”数量＞4，你进入“结茧”状态，重生时恢复初始状态。此技能仅生效一次</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>化茧</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Cocooning</t>
-  </si>
-  <si>
     <t>时钟拨回起点，让我们重新演绎这场闹剧</t>
   </si>
   <si>
-    <t>当你生命值为≤0时，若场上有虚空兽存在，一只虚空兽立刻变为“茧”，你借此茧重生</t>
-  </si>
-  <si>
-    <t>时序逆转</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Time Reversal</t>
-  </si>
-  <si>
     <t>（低吼声……）</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1574,13 +1553,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>扭曲时空，令时间之手对玩家追击一次“砍”，记忆之手对玩家追击一次“给枪”。若二者资源不足以发动，消耗所有资源，依然发动。</t>
-  </si>
-  <si>
-    <t>吞噬星空</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Devour the Stars</t>
   </si>
   <si>
@@ -1604,17 +1576,6 @@
   <si>
     <t>我的，不可置疑</t>
     <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>下一回合，你使用“补给”类行动时，额外获得3点刀剑与2点子弹。下一回合，你使用非“补给”类行动时，刷新该技能CD。</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>威压</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Intimidation</t>
   </si>
   <si>
     <t>力不竭、战不止</t>
@@ -1810,9 +1771,6 @@
   </si>
   <si>
     <t>Bloodborne Rebirth</t>
-  </si>
-  <si>
-    <t>当你防御或反制成功时，你下回合攻击力+1</t>
   </si>
   <si>
     <t>突跃反击</t>
@@ -1950,9 +1908,6 @@
   </si>
   <si>
     <t>Blazing Dance</t>
-  </si>
-  <si>
-    <t>接下来的3个回合内，你可以在追击阶段仅一次使用一张免费的“刺”，追击后进入CD</t>
   </si>
   <si>
     <t>短匕</t>
@@ -2201,6 +2156,58 @@
     <t>下回合你的所有伤害+1，攻击力+0.5</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>回合开始时发动，若有足够的资源，令时间之手对玩家追击一次“砍”，或记忆之手对玩家追击一次“给枪”。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>吞噬星空（修改）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Time Reversal</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>倒转时空</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>当你生命值为≤0时，若场上有虚空兽存在，一只虚空兽立刻变为“茧”，你借此茧重生</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Time Fasting</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>时间加速</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有友方下一回合的行动将会额外执行一次</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Time Distortion</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>时空扭曲</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>下一回合，所有人将额外执行一次这轮的行动。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>你可以在追击阶段仅一次使用一张免费的“刺”，追击后进入CD</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>当你防御或反制成功时，你下回合攻击力+1.5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -2218,6 +2225,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -2781,7 +2789,7 @@
     </row>
     <row r="3" spans="1:18" ht="25" x14ac:dyDescent="0.5">
       <c r="A3" s="32" t="s">
-        <v>517</v>
+        <v>504</v>
       </c>
       <c r="Q3" s="31"/>
       <c r="R3" s="31"/>
@@ -2792,56 +2800,56 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="30" t="s">
-        <v>516</v>
+        <v>503</v>
       </c>
       <c r="Q5" s="31"/>
       <c r="R5" s="31"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="30" t="s">
-        <v>515</v>
+        <v>502</v>
       </c>
       <c r="Q6" s="31"/>
       <c r="R6" s="31"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
-        <v>514</v>
+        <v>501</v>
       </c>
       <c r="Q7" s="31"/>
       <c r="R7" s="31"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="30" t="s">
-        <v>513</v>
+        <v>500</v>
       </c>
       <c r="Q8" s="31"/>
       <c r="R8" s="31"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="30" t="s">
-        <v>512</v>
+        <v>499</v>
       </c>
       <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="30" t="s">
-        <v>511</v>
+        <v>498</v>
       </c>
       <c r="Q10" s="31"/>
       <c r="R10" s="31"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="30" t="s">
-        <v>510</v>
+        <v>497</v>
       </c>
       <c r="Q11" s="31"/>
       <c r="R11" s="31"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="30" t="s">
-        <v>509</v>
+        <v>496</v>
       </c>
       <c r="Q12" s="31"/>
       <c r="R12" s="31"/>
@@ -3232,19 +3240,19 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
-        <v>406</v>
+        <v>395</v>
       </c>
       <c r="B1" s="28" t="s">
-        <v>508</v>
+        <v>495</v>
       </c>
       <c r="C1" s="28" t="s">
-        <v>507</v>
+        <v>494</v>
       </c>
       <c r="D1" s="28" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="E1" s="29" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
@@ -3260,17 +3268,17 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>506</v>
+        <v>493</v>
       </c>
       <c r="C2" s="23" t="str">
         <f t="shared" ref="C2:C10" si="0">B2</f>
         <v>Diving</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>505</v>
+        <v>492</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>504</v>
+        <v>491</v>
       </c>
       <c r="F2" s="23"/>
       <c r="G2" s="23"/>
@@ -3286,17 +3294,17 @@
         <v>2</v>
       </c>
       <c r="B3" s="21" t="s">
-        <v>503</v>
+        <v>490</v>
       </c>
       <c r="C3" s="21" t="str">
         <f t="shared" si="0"/>
         <v>Stunned</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>502</v>
+        <v>489</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>501</v>
+        <v>488</v>
       </c>
       <c r="R3" s="27"/>
       <c r="S3" s="27"/>
@@ -3306,17 +3314,17 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>500</v>
+        <v>487</v>
       </c>
       <c r="C4" s="23" t="str">
         <f t="shared" si="0"/>
         <v>Invincible</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>499</v>
+        <v>486</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>498</v>
+        <v>485</v>
       </c>
       <c r="F4" s="23"/>
       <c r="G4" s="23"/>
@@ -3334,17 +3342,17 @@
         <v>4</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>497</v>
+        <v>484</v>
       </c>
       <c r="C5" s="25" t="str">
         <f t="shared" si="0"/>
         <v>Critical</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>496</v>
+        <v>483</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>495</v>
+        <v>482</v>
       </c>
       <c r="F5" s="25"/>
       <c r="G5" s="25"/>
@@ -3362,17 +3370,17 @@
         <v>5</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>494</v>
+        <v>481</v>
       </c>
       <c r="C6" s="23" t="str">
         <f t="shared" si="0"/>
         <v>Slowed</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>493</v>
+        <v>480</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>492</v>
+        <v>479</v>
       </c>
       <c r="F6" s="23"/>
       <c r="G6" s="23"/>
@@ -3390,17 +3398,17 @@
         <v>6</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>491</v>
+        <v>478</v>
       </c>
       <c r="C7" s="21" t="str">
         <f t="shared" si="0"/>
         <v>Burning</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>490</v>
+        <v>477</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>489</v>
+        <v>476</v>
       </c>
       <c r="R7" s="27"/>
       <c r="S7" s="27"/>
@@ -3410,17 +3418,17 @@
         <v>7</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>488</v>
+        <v>475</v>
       </c>
       <c r="C8" s="23" t="str">
         <f t="shared" si="0"/>
         <v>Cocooned</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>487</v>
+        <v>474</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>486</v>
+        <v>473</v>
       </c>
       <c r="F8" s="23"/>
       <c r="G8" s="23"/>
@@ -3438,17 +3446,17 @@
         <v>8</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>485</v>
+        <v>472</v>
       </c>
       <c r="C9" s="25" t="str">
         <f t="shared" si="0"/>
         <v>Crystallized</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>484</v>
+        <v>471</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>483</v>
+        <v>470</v>
       </c>
       <c r="F9" s="25"/>
       <c r="G9" s="25"/>
@@ -3466,17 +3474,17 @@
         <v>9</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>482</v>
+        <v>469</v>
       </c>
       <c r="C10" s="23" t="str">
         <f t="shared" si="0"/>
         <v>Bleeding</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>481</v>
+        <v>468</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>480</v>
+        <v>467</v>
       </c>
       <c r="F10" s="23"/>
       <c r="G10" s="23"/>
@@ -3564,34 +3572,34 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>479</v>
+        <v>466</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="J1" s="18" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
       <c r="K1" s="18"/>
       <c r="L1" s="19"/>
@@ -3606,14 +3614,14 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>478</v>
+        <v>465</v>
       </c>
       <c r="B2" s="15" t="str">
         <f t="shared" ref="B2:B26" si="0">A2</f>
         <v>Rapid Supply</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>477</v>
+        <v>464</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>29</v>
@@ -3621,10 +3629,10 @@
       <c r="E2" s="15"/>
       <c r="F2" s="15"/>
       <c r="G2" s="13" t="s">
-        <v>476</v>
+        <v>463</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I2" s="15" t="s">
         <v>0</v>
@@ -3645,14 +3653,14 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
-        <v>475</v>
+        <v>462</v>
       </c>
       <c r="B3" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Candlelight Sanctuary</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>474</v>
+        <v>461</v>
       </c>
       <c r="D3" s="16" t="s">
         <v>29</v>
@@ -3664,10 +3672,10 @@
         <v>1</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>473</v>
+        <v>460</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I3" s="16" t="s">
         <v>0</v>
@@ -3688,14 +3696,14 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>472</v>
+        <v>459</v>
       </c>
       <c r="B4" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Feedback</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>471</v>
+        <v>458</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>3</v>
@@ -3703,10 +3711,10 @@
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
       <c r="G4" s="13" t="s">
-        <v>470</v>
+        <v>457</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I4" s="15" t="s">
         <v>169</v>
@@ -3746,10 +3754,10 @@
         <v>2</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>521</v>
+        <v>508</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I5" s="16" t="s">
         <v>6</v>
@@ -3770,14 +3778,14 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
-        <v>469</v>
+        <v>456</v>
       </c>
       <c r="B6" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Reverse Decision</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>468</v>
+        <v>455</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>3</v>
@@ -3789,10 +3797,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>522</v>
+        <v>509</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I6" s="15" t="s">
         <v>6</v>
@@ -3813,14 +3821,14 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>467</v>
+        <v>454</v>
       </c>
       <c r="B7" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Bloody Brawl</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>466</v>
+        <v>453</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>29</v>
@@ -3828,10 +3836,10 @@
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="14" t="s">
-        <v>523</v>
+        <v>510</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I7" s="16" t="s">
         <v>20</v>
@@ -3852,14 +3860,14 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
-        <v>465</v>
+        <v>452</v>
       </c>
       <c r="B8" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Battle on All Sides</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>464</v>
+        <v>451</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>3</v>
@@ -3867,10 +3875,10 @@
       <c r="E8" s="15"/>
       <c r="F8" s="15"/>
       <c r="G8" s="13" t="s">
-        <v>519</v>
+        <v>506</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I8" s="15" t="s">
         <v>6</v>
@@ -3891,14 +3899,14 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
-        <v>463</v>
+        <v>450</v>
       </c>
       <c r="B9" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Short Dagger</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>462</v>
+        <v>449</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>29</v>
@@ -3906,10 +3914,10 @@
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="14" t="s">
-        <v>461</v>
+        <v>522</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I9" s="16" t="s">
         <v>6</v>
@@ -3930,14 +3938,14 @@
     </row>
     <row r="10" spans="1:20" ht="26" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>460</v>
+        <v>448</v>
       </c>
       <c r="B10" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Blazing Dance</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>459</v>
+        <v>447</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>3</v>
@@ -3945,10 +3953,10 @@
       <c r="E10" s="15"/>
       <c r="F10" s="15"/>
       <c r="G10" s="13" t="s">
-        <v>520</v>
+        <v>507</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I10" s="15" t="s">
         <v>6</v>
@@ -3969,14 +3977,14 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>458</v>
+        <v>446</v>
       </c>
       <c r="B11" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Poisoned Sword</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>457</v>
+        <v>445</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>3</v>
@@ -3984,10 +3992,10 @@
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="14" t="s">
-        <v>456</v>
+        <v>444</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I11" s="16" t="s">
         <v>6</v>
@@ -4008,14 +4016,14 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
-        <v>455</v>
+        <v>443</v>
       </c>
       <c r="B12" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Mist Shadow Sword</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>454</v>
+        <v>442</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>3</v>
@@ -4023,10 +4031,10 @@
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="13" t="s">
-        <v>453</v>
+        <v>441</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>452</v>
+        <v>440</v>
       </c>
       <c r="I12" s="15" t="s">
         <v>6</v>
@@ -4047,14 +4055,14 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
-        <v>451</v>
+        <v>439</v>
       </c>
       <c r="B13" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Fight to the Death</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>450</v>
+        <v>438</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>3</v>
@@ -4062,10 +4070,10 @@
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="14" t="s">
-        <v>449</v>
+        <v>437</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I13" s="16" t="s">
         <v>6</v>
@@ -4086,14 +4094,14 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="15" t="s">
-        <v>448</v>
+        <v>436</v>
       </c>
       <c r="B14" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Attract Misfortune</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>447</v>
+        <v>435</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>23</v>
@@ -4105,10 +4113,10 @@
         <v>2</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>446</v>
+        <v>434</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I14" s="15" t="s">
         <v>169</v>
@@ -4129,14 +4137,14 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
-        <v>445</v>
+        <v>433</v>
       </c>
       <c r="B15" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Painful Thorns</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>444</v>
+        <v>432</v>
       </c>
       <c r="D15" s="16" t="s">
         <v>29</v>
@@ -4144,13 +4152,13 @@
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
       <c r="G15" s="14" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>442</v>
+        <v>430</v>
       </c>
       <c r="J15" s="16">
         <v>5</v>
@@ -4168,14 +4176,14 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="15" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="B16" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Crystal Armor</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>3</v>
@@ -4183,10 +4191,10 @@
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
       <c r="G16" s="13" t="s">
-        <v>439</v>
+        <v>427</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I16" s="15" t="s">
         <v>6</v>
@@ -4207,14 +4215,14 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
-        <v>438</v>
+        <v>426</v>
       </c>
       <c r="B17" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Purification Amulet</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>3</v>
@@ -4222,10 +4230,10 @@
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
       <c r="G17" s="14" t="s">
-        <v>436</v>
+        <v>424</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I17" s="16" t="s">
         <v>6</v>
@@ -4246,14 +4254,14 @@
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="15" t="s">
-        <v>435</v>
+        <v>423</v>
       </c>
       <c r="B18" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Forest's Breath</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>29</v>
@@ -4265,13 +4273,13 @@
         <v>3</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>433</v>
+        <v>421</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="J18" s="15">
         <v>0</v>
@@ -4289,14 +4297,14 @@
     </row>
     <row r="19" spans="1:20" ht="26" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
-        <v>432</v>
+        <v>420</v>
       </c>
       <c r="B19" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Cursed Soul's Whisper</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>431</v>
+        <v>419</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>29</v>
@@ -4308,10 +4316,10 @@
         <v>2</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>430</v>
+        <v>418</v>
       </c>
       <c r="H19" s="16" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I19" s="16" t="s">
         <v>26</v>
@@ -4332,14 +4340,14 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="15" t="s">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="B20" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Enlighten</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>428</v>
+        <v>416</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>29</v>
@@ -4347,13 +4355,13 @@
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
       <c r="G20" s="13" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="J20" s="15">
         <v>3</v>
@@ -4371,14 +4379,14 @@
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="B21" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Leap Counter</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>3</v>
@@ -4386,10 +4394,10 @@
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
       <c r="G21" s="14" t="s">
-        <v>424</v>
+        <v>523</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I21" s="16" t="s">
         <v>6</v>
@@ -4410,14 +4418,14 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="15" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="B22" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Bloodborne Rebirth</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>3</v>
@@ -4429,10 +4437,10 @@
         <v>1</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I22" s="15" t="s">
         <v>6</v>
@@ -4453,14 +4461,14 @@
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="B23" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Flawless Defense</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>29</v>
@@ -4472,10 +4480,10 @@
         <v>2</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="H23" s="16" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I23" s="16" t="s">
         <v>6</v>
@@ -4496,14 +4504,14 @@
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="15" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="B24" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Territorial Imprisonment</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>29</v>
@@ -4515,10 +4523,10 @@
         <v>3</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>415</v>
+        <v>404</v>
       </c>
       <c r="H24" s="15" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="I24" s="15" t="s">
         <v>6</v>
@@ -4539,14 +4547,14 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
       <c r="B25" s="16" t="str">
         <f t="shared" si="0"/>
         <v>Immovable as a Bell</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="D25" s="16" t="s">
         <v>3</v>
@@ -4554,10 +4562,10 @@
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
       <c r="G25" s="14" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="H25" s="16" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I25" s="16" t="s">
         <v>6</v>
@@ -4578,14 +4586,14 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="15" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="B26" s="15" t="str">
         <f t="shared" si="0"/>
         <v>Charging Shield</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>409</v>
+        <v>398</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>3</v>
@@ -4593,10 +4601,10 @@
       <c r="E26" s="15"/>
       <c r="F26" s="15"/>
       <c r="G26" s="13" t="s">
-        <v>408</v>
+        <v>397</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="I26" s="15" t="s">
         <v>6</v>
@@ -4968,43 +4976,43 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>406</v>
+        <v>395</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>405</v>
+        <v>394</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>404</v>
+        <v>393</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>403</v>
+        <v>392</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>399</v>
+        <v>388</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>398</v>
+        <v>387</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>397</v>
+        <v>386</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>396</v>
+        <v>385</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>395</v>
+        <v>384</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>394</v>
+        <v>383</v>
       </c>
       <c r="N1" s="7"/>
       <c r="O1" s="8"/>
@@ -5025,14 +5033,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>393</v>
+        <v>382</v>
       </c>
       <c r="C2" s="3" t="str">
         <f t="shared" ref="C2:C33" si="0">B2</f>
         <v>Save Me!!!</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>3</v>
@@ -5044,11 +5052,11 @@
         <v>1</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="3" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>0</v>
@@ -5078,14 +5086,14 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="C3" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Toy Assembly Line</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>388</v>
+        <v>377</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>29</v>
@@ -5095,11 +5103,11 @@
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="6" t="s">
-        <v>387</v>
+        <v>376</v>
       </c>
       <c r="I3" s="6"/>
       <c r="J3" s="5" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="K3" s="5"/>
       <c r="L3" s="5">
@@ -5127,14 +5135,14 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>385</v>
+        <v>374</v>
       </c>
       <c r="C4" s="3" t="str">
         <f t="shared" si="0"/>
         <v>Castle Guardian</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>384</v>
+        <v>373</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>3</v>
@@ -5146,11 +5154,11 @@
         <v>1</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>383</v>
+        <v>372</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" s="3" t="s">
-        <v>382</v>
+        <v>371</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>0</v>
@@ -5180,14 +5188,14 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
       <c r="C5" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Fight Again</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>3</v>
@@ -5199,11 +5207,11 @@
         <v>1</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="5" t="s">
-        <v>378</v>
+        <v>367</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>6</v>
@@ -5233,14 +5241,14 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>377</v>
+        <v>366</v>
       </c>
       <c r="C6" s="3" t="str">
         <f t="shared" si="0"/>
         <v>Waraxe Dance</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>23</v>
@@ -5250,11 +5258,11 @@
       </c>
       <c r="G6" s="3"/>
       <c r="H6" s="4" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" s="3" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>286</v>
@@ -5284,14 +5292,14 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>373</v>
+        <v>519</v>
       </c>
       <c r="C7" s="5" t="str">
         <f t="shared" si="0"/>
-        <v>Intimidation</v>
+        <v>Time Distortion</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>372</v>
+        <v>520</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>29</v>
@@ -5301,11 +5309,11 @@
       </c>
       <c r="G7" s="5"/>
       <c r="H7" s="6" t="s">
-        <v>371</v>
+        <v>521</v>
       </c>
       <c r="I7" s="6"/>
       <c r="J7" s="5" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>6</v>
@@ -5335,14 +5343,14 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="C8" s="3" t="str">
         <f t="shared" si="0"/>
         <v>Void Servant</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>29</v>
@@ -5352,14 +5360,14 @@
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="4" t="s">
-        <v>367</v>
+        <v>359</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" s="3" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="L8" s="3">
         <v>2</v>
@@ -5386,14 +5394,14 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="C9" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Devour the Stars</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>363</v>
+        <v>512</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>23</v>
@@ -5403,14 +5411,14 @@
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="6" t="s">
-        <v>362</v>
+        <v>511</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="5" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="L9" s="5">
         <v>4</v>
@@ -5437,14 +5445,14 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="C10" s="3" t="str">
         <f t="shared" si="0"/>
         <v>Morphing Remains</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>3</v>
@@ -5454,11 +5462,11 @@
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="4" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="3" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>0</v>
@@ -5488,14 +5496,14 @@
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="C11" s="5" t="str">
         <f t="shared" si="0"/>
         <v>Charge</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>3</v>
@@ -5507,11 +5515,11 @@
         <v>1</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
       <c r="I11" s="6"/>
       <c r="J11" s="5" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>6</v>
@@ -5541,14 +5549,14 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>351</v>
+        <v>516</v>
       </c>
       <c r="C12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Time Reversal</v>
+        <f>B12</f>
+        <v>Time Fasting</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>350</v>
+        <v>517</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>3</v>
@@ -5560,11 +5568,11 @@
         <v>1</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>349</v>
+        <v>518</v>
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="3" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>0</v>
@@ -5589,19 +5597,19 @@
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
     </row>
-    <row r="13" spans="1:26" ht="26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>347</v>
+        <v>513</v>
       </c>
       <c r="C13" s="5" t="str">
-        <f t="shared" si="0"/>
-        <v>Cocooning</v>
+        <f>B13</f>
+        <v>Time Reversal</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>346</v>
+        <v>514</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>3</v>
@@ -5613,7 +5621,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>345</v>
+        <v>515</v>
       </c>
       <c r="I13" s="6"/>
       <c r="J13" s="5" t="s">
@@ -5717,7 +5725,7 @@
         <v>337</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>518</v>
+        <v>505</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="5" t="s">
@@ -6680,7 +6688,7 @@
         <v>261</v>
       </c>
       <c r="C34" s="3" t="str">
-        <f t="shared" ref="C34:C65" si="1">B34</f>
+        <f t="shared" ref="C34:C54" si="1">B34</f>
         <v>Water Warding Incantation</v>
       </c>
       <c r="D34" s="3" t="s">

</xml_diff>